<commit_message>
min score from 0.35 to 0.5
</commit_message>
<xml_diff>
--- a/docs/results.xlsx
+++ b/docs/results.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\babar\Learning Path\Machine learning Engineering\RAG\Project 01\local-rag\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E9BDAE9-9E8D-45EA-91E0-C75AA0DC3DFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADAF5843-6800-499C-9270-4217D1E6CEDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -434,7 +434,8 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.7109375" customWidth="1"/>
-    <col min="2" max="3" width="23" customWidth="1"/>
+    <col min="2" max="2" width="23" customWidth="1"/>
+    <col min="3" max="3" width="28.5703125" customWidth="1"/>
     <col min="4" max="4" width="38.7109375" customWidth="1"/>
     <col min="5" max="5" width="23.28515625" customWidth="1"/>
     <col min="6" max="6" width="27" customWidth="1"/>

</xml_diff>